<commit_message>
Feat: end-to-end 3-class fine-tuning + resumable continuation
- src/training/finetune_3class.py: loads the latest 3-class head_full.keras
  and runs Stage-2 fine-tuning (unfreeze last 20 backbone layers, lr=1e-5)
  against data/splits_3class/ with the ResourceLogger callback.
- src/training/finetune_3class_continue.py: resumes from the latest
  fine_tuned.keras, runs more epochs, and merges new history + resources
  into the original Training<N> dir with shifted epoch indices so the
  Excel sheet shows one continuous curve.
- src/export/metrics_to_excel.py: collect() now returns the latest of
  *each* stage (head + finetune) so the workbook reflects both.
- outputs/Training13/{history,resources}_finetune.json: 10 merged epochs,
  best val_acc 0.976 @ epoch 10, best val_loss 0.086; thermal peaked at
  85.9 C (above Pi 5 hard-throttle at 85 C).
- outputs/training_metrics.xlsx: regenerated with both stages.
- .gitignore: exclude data/splits_3class/ (symlinks to data/splits/).
</commit_message>
<xml_diff>
--- a/outputs/training_metrics.xlsx
+++ b/outputs/training_metrics.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Resources" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Training12_Stage1_Head_v2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Training13_Stage2_FineTune" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -504,6 +505,42 @@
       </c>
       <c r="J2" t="n">
         <v>0.02218616008758545</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Training13</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Stage2_FineTune</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.9755747318267822</v>
+      </c>
+      <c r="E3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.9755747318267822</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.08631157875061035</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.9620953798294067</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.1038081273436546</v>
+      </c>
+      <c r="J3" t="n">
+        <v>-0.01347935199737549</v>
       </c>
     </row>
   </sheetData>
@@ -517,7 +554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -630,6 +667,51 @@
       </c>
       <c r="M2" t="n">
         <v>62.8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Training13</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Stage2_FineTune</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1038.866</v>
+      </c>
+      <c r="E3" t="n">
+        <v>103.8866</v>
+      </c>
+      <c r="F3" t="n">
+        <v>70.476</v>
+      </c>
+      <c r="G3" t="n">
+        <v>90</v>
+      </c>
+      <c r="H3" t="n">
+        <v>26.411</v>
+      </c>
+      <c r="I3" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="J3" t="n">
+        <v>2.2318</v>
+      </c>
+      <c r="K3" t="n">
+        <v>2.495</v>
+      </c>
+      <c r="L3" t="n">
+        <v>77.414</v>
+      </c>
+      <c r="M3" t="n">
+        <v>85.90000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -1149,4 +1231,565 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>epoch</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>val_accuracy</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>val_loss</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>epoch_seconds</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>cpu_percent_mean</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>cpu_percent_max</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>ram_percent_mean</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>ram_percent_peak</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>ram_used_gb_mean</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ram_used_gb_peak</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>temp_c_mean</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>temp_c_max</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>samples_per_epoch</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.9369676113128662</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.9583333134651184</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.1899844110012054</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.1380274742841721</v>
+      </c>
+      <c r="F2" t="n">
+        <v>200.332</v>
+      </c>
+      <c r="G2" t="n">
+        <v>45.39</v>
+      </c>
+      <c r="H2" t="n">
+        <v>89.09999999999999</v>
+      </c>
+      <c r="I2" t="n">
+        <v>21.53</v>
+      </c>
+      <c r="J2" t="n">
+        <v>27</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1.819</v>
+      </c>
+      <c r="L2" t="n">
+        <v>2.282</v>
+      </c>
+      <c r="M2" t="n">
+        <v>63.72</v>
+      </c>
+      <c r="N2" t="n">
+        <v>76</v>
+      </c>
+      <c r="O2" t="n">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.9527257084846497</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.9554597735404968</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.1387090981006622</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.1439083963632584</v>
+      </c>
+      <c r="F3" t="n">
+        <v>120.357</v>
+      </c>
+      <c r="G3" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="H3" t="n">
+        <v>90</v>
+      </c>
+      <c r="I3" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="J3" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="K3" t="n">
+        <v>2.136</v>
+      </c>
+      <c r="L3" t="n">
+        <v>2.312</v>
+      </c>
+      <c r="M3" t="n">
+        <v>68.58</v>
+      </c>
+      <c r="N3" t="n">
+        <v>79.8</v>
+      </c>
+      <c r="O3" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0.9471890926361084</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.9568965435028076</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.1519994735717773</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.1333447992801666</v>
+      </c>
+      <c r="F4" t="n">
+        <v>66.476</v>
+      </c>
+      <c r="G4" t="n">
+        <v>85.48999999999999</v>
+      </c>
+      <c r="H4" t="n">
+        <v>88.3</v>
+      </c>
+      <c r="I4" t="n">
+        <v>27.57</v>
+      </c>
+      <c r="J4" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="K4" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="L4" t="n">
+        <v>2.396</v>
+      </c>
+      <c r="M4" t="n">
+        <v>80.59999999999999</v>
+      </c>
+      <c r="N4" t="n">
+        <v>84.2</v>
+      </c>
+      <c r="O4" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.9531516432762146</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.959770143032074</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.141852393746376</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.1213065385818481</v>
+      </c>
+      <c r="F5" t="n">
+        <v>95.97499999999999</v>
+      </c>
+      <c r="G5" t="n">
+        <v>64.44</v>
+      </c>
+      <c r="H5" t="n">
+        <v>90</v>
+      </c>
+      <c r="I5" t="n">
+        <v>27.65</v>
+      </c>
+      <c r="J5" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="K5" t="n">
+        <v>2.337</v>
+      </c>
+      <c r="L5" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="M5" t="n">
+        <v>80.47</v>
+      </c>
+      <c r="N5" t="n">
+        <v>84.8</v>
+      </c>
+      <c r="O5" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0.9574105739593506</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.9640804529190063</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.1237899288535118</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.1125743165612221</v>
+      </c>
+      <c r="F6" t="n">
+        <v>69.69499999999999</v>
+      </c>
+      <c r="G6" t="n">
+        <v>85.42</v>
+      </c>
+      <c r="H6" t="n">
+        <v>88.90000000000001</v>
+      </c>
+      <c r="I6" t="n">
+        <v>27.88</v>
+      </c>
+      <c r="J6" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="K6" t="n">
+        <v>2.356</v>
+      </c>
+      <c r="L6" t="n">
+        <v>2.467</v>
+      </c>
+      <c r="M6" t="n">
+        <v>83.27</v>
+      </c>
+      <c r="N6" t="n">
+        <v>84.8</v>
+      </c>
+      <c r="O6" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.9531516432762146</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.9626436829566956</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.1321223974227905</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.1105362325906754</v>
+      </c>
+      <c r="F7" t="n">
+        <v>201.568</v>
+      </c>
+      <c r="G7" t="n">
+        <v>45.71</v>
+      </c>
+      <c r="H7" t="n">
+        <v>88.40000000000001</v>
+      </c>
+      <c r="I7" t="n">
+        <v>21.54</v>
+      </c>
+      <c r="J7" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1.821</v>
+      </c>
+      <c r="L7" t="n">
+        <v>2.249</v>
+      </c>
+      <c r="M7" t="n">
+        <v>66</v>
+      </c>
+      <c r="N7" t="n">
+        <v>78.2</v>
+      </c>
+      <c r="O7" t="n">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.9552810788154602</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.9640804529190063</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.1131835207343102</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.105962947010994</v>
+      </c>
+      <c r="F8" t="n">
+        <v>66.765</v>
+      </c>
+      <c r="G8" t="n">
+        <v>85.03</v>
+      </c>
+      <c r="H8" t="n">
+        <v>89.2</v>
+      </c>
+      <c r="I8" t="n">
+        <v>27.81</v>
+      </c>
+      <c r="J8" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="L8" t="n">
+        <v>2.442</v>
+      </c>
+      <c r="M8" t="n">
+        <v>80.94</v>
+      </c>
+      <c r="N8" t="n">
+        <v>84.8</v>
+      </c>
+      <c r="O8" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.9578364491462708</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.9698275923728943</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.1082411929965019</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.09996028244495392</v>
+      </c>
+      <c r="F9" t="n">
+        <v>69.14</v>
+      </c>
+      <c r="G9" t="n">
+        <v>85.36</v>
+      </c>
+      <c r="H9" t="n">
+        <v>88.40000000000001</v>
+      </c>
+      <c r="I9" t="n">
+        <v>28.23</v>
+      </c>
+      <c r="J9" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2.385</v>
+      </c>
+      <c r="L9" t="n">
+        <v>2.462</v>
+      </c>
+      <c r="M9" t="n">
+        <v>83.41</v>
+      </c>
+      <c r="N9" t="n">
+        <v>85.3</v>
+      </c>
+      <c r="O9" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.9629471898078918</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.9741379022598267</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.09774375706911087</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.09146703779697418</v>
+      </c>
+      <c r="F10" t="n">
+        <v>69.90300000000001</v>
+      </c>
+      <c r="G10" t="n">
+        <v>84.70999999999999</v>
+      </c>
+      <c r="H10" t="n">
+        <v>88.7</v>
+      </c>
+      <c r="I10" t="n">
+        <v>28.31</v>
+      </c>
+      <c r="J10" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="K10" t="n">
+        <v>2.392</v>
+      </c>
+      <c r="L10" t="n">
+        <v>2.495</v>
+      </c>
+      <c r="M10" t="n">
+        <v>83.56999999999999</v>
+      </c>
+      <c r="N10" t="n">
+        <v>85.90000000000001</v>
+      </c>
+      <c r="O10" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.9620953798294067</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.9755747318267822</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.1038081273436546</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.08631157875061035</v>
+      </c>
+      <c r="F11" t="n">
+        <v>78.655</v>
+      </c>
+      <c r="G11" t="n">
+        <v>76.70999999999999</v>
+      </c>
+      <c r="H11" t="n">
+        <v>87.90000000000001</v>
+      </c>
+      <c r="I11" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="J11" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="K11" t="n">
+        <v>2.392</v>
+      </c>
+      <c r="L11" t="n">
+        <v>2.484</v>
+      </c>
+      <c r="M11" t="n">
+        <v>83.58</v>
+      </c>
+      <c r="N11" t="n">
+        <v>85.90000000000001</v>
+      </c>
+      <c r="O11" t="n">
+        <v>78</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>